<commit_message>
feat: add support for 'select_missing_words' question type and integrate MathJax for LaTeX rendering
</commit_message>
<xml_diff>
--- a/public/templates/moodle_xml_sheet_templates.xlsx
+++ b/public/templates/moodle_xml_sheet_templates.xlsx
@@ -2,18 +2,19 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Allowed_Values" sheetId="1" r:id="R2c26b11e7b214ff6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Huong_Dan" sheetId="2" r:id="Rf6b87eecbeb040f2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_Single_Choice" sheetId="3" r:id="R4a184a2d8c924971"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_Multiple_Choice" sheetId="4" r:id="Rc2230f5a847e4075"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_TrueFalse" sheetId="5" r:id="Rd7829a192a8b4ae4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_ShortAnswer" sheetId="6" r:id="Rcde848e960024c17"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_Numerical" sheetId="7" r:id="Rb6e1e16865c24326"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_Matching" sheetId="8" r:id="Re5119bd82ec04c70"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_DragDrop_Text" sheetId="9" r:id="R0dee2550e4d04c58"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_Essay_Desc_Cloze" sheetId="10" r:id="R23aa4f189fe14b4d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_Reading_Passage" sheetId="11" r:id="Rf6426542126a4cd6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_Full_Demo" sheetId="12" r:id="Rbb7f6ab701fd4f93"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Allowed_Values" sheetId="1" r:id="R8908574161f74c05"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Huong_Dan" sheetId="2" r:id="R756b5b2b5d164d69"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_Single_Choice" sheetId="3" r:id="R09164b6849ea46fa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_Multiple_Choice" sheetId="4" r:id="R4c45caa7cd3b4b63"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_TrueFalse" sheetId="5" r:id="R92014d83ad394f0b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_ShortAnswer" sheetId="6" r:id="R1e7eddc003fc46ef"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_Numerical" sheetId="7" r:id="R729db0cace884da7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_Matching" sheetId="8" r:id="Rb73f3abeb1c94532"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_DragDrop_Text" sheetId="9" r:id="R70b91db75ff949b9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_Essay_Desc_Cloze" sheetId="10" r:id="R2a9cae92b9344d19"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_Reading_Passage" sheetId="11" r:id="Rf064df3fa29a410e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_Full_Demo" sheetId="12" r:id="Rbb757e08f9334aae"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_Select_Missing_Words" sheetId="13" r:id="R1ca4d755589044c4"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -42,7 +43,7 @@
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="4">
+  <x:fills count="7">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -59,15 +60,44 @@
         <x:fgColor rgb="FFDBEAFE"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF2445B6"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF2445B6"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF2445B6"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
-  <x:borders count="2">
+  <x:borders count="3">
     <x:border/>
     <x:border/>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:bottom>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="22">
+  <x:cellXfs count="30">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -114,11 +144,47 @@
     <x:xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
 </x:styleSheet>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="SelectMissingWordsTable" displayName="SelectMissingWordsTable" ref="A1:J4" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="10">
+    <x:tableColumn id="1" name="category"/>
+    <x:tableColumn id="2" name="question_id"/>
+    <x:tableColumn id="3" name="type"/>
+    <x:tableColumn id="4" name="question_name"/>
+    <x:tableColumn id="5" name="question_text"/>
+    <x:tableColumn id="6" name="drag_no"/>
+    <x:tableColumn id="7" name="drag_text"/>
+    <x:tableColumn id="8" name="group"/>
+    <x:tableColumn id="9" name="explanation"/>
+    <x:tableColumn id="10" name="grade"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -164,9 +230,9 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri"/>
-        <a:ea typeface="Calibri"/>
-        <a:cs typeface="Calibri"/>
+        <a:latin typeface="Calibri Light"/>
+        <a:ea typeface="Calibri Light"/>
+        <a:cs typeface="Calibri Light"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -410,6 +476,16 @@
         <x:v>Embedded answers</x:v>
       </x:c>
     </x:row>
+    <x:row r="12">
+      <x:c r="A12" t="str">
+        <x:v>select_missing_words</x:v>
+      </x:c>
+      <x:c r="B12"/>
+      <x:c r="C12"/>
+      <x:c r="D12" t="str">
+        <x:v>Chọn từ/cụm từ còn thiếu, Moodle type gapselect</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -517,10 +593,32 @@
         <x:v>2</x:v>
       </x:c>
     </x:row>
+    <x:row r="5" ht="42" customHeight="1">
+      <x:c r="A5" t="str">
+        <x:v>TSA/Toán</x:v>
+      </x:c>
+      <x:c r="B5" t="str">
+        <x:v>C002</x:v>
+      </x:c>
+      <x:c r="C5" t="str">
+        <x:v>cloze</x:v>
+      </x:c>
+      <x:c r="D5" t="str">
+        <x:v>Cloze LaTeX</x:v>
+      </x:c>
+      <x:c r="E5" s="12" t="str">
+        <x:v>Giải phương trình $x^2=4$: {1:SHORTANSWER:=2~=-2}. Hằng đẳng thức: \(a^2-b^2=(a-b)(a+b)\).</x:v>
+      </x:c>
+      <x:c r="F5"/>
+      <x:c r="G5"/>
+      <x:c r="H5" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:dataValidations count="1">
     <x:dataValidation type="list" sqref="C2:C200">
-      <x:formula1>_Allowed_Values!$A$2:$A$11</x:formula1>
+      <x:formula1>_Allowed_Values!$A$2:$A$12</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -665,7 +763,7 @@
   </x:sheetData>
   <x:dataValidations count="1">
     <x:dataValidation type="list" sqref="E2:E200">
-      <x:formula1>_Allowed_Values!$A$2:$A$11</x:formula1>
+      <x:formula1>_Allowed_Values!$A$2:$A$12</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1283,16 +1381,299 @@
       </x:c>
       <x:c r="V14" s="14" t="str"/>
     </x:row>
+    <x:row r="15" ht="30" customHeight="1">
+      <x:c r="A15" t="str">
+        <x:v>Demo</x:v>
+      </x:c>
+      <x:c r="B15" t="str">
+        <x:v>SMW001</x:v>
+      </x:c>
+      <x:c r="C15" t="str">
+        <x:v>select_missing_words</x:v>
+      </x:c>
+      <x:c r="D15" t="str">
+        <x:v>SelectMissingWords</x:v>
+      </x:c>
+      <x:c r="E15" s="12" t="str">
+        <x:v>The derivative of $x^2$ is [[1]].</x:v>
+      </x:c>
+      <x:c r="F15"/>
+      <x:c r="G15"/>
+      <x:c r="H15"/>
+      <x:c r="I15"/>
+      <x:c r="J15"/>
+      <x:c r="K15"/>
+      <x:c r="L15"/>
+      <x:c r="M15"/>
+      <x:c r="N15" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="O15" t="str">
+        <x:v>2x</x:v>
+      </x:c>
+      <x:c r="P15" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="Q15" t="str">
+        <x:v>FALSE</x:v>
+      </x:c>
+      <x:c r="R15"/>
+      <x:c r="S15"/>
+      <x:c r="T15"/>
+      <x:c r="U15" t="str">
+        <x:v>LaTeX trong preview sẽ được MathJax render.</x:v>
+      </x:c>
+      <x:c r="V15" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="30" customHeight="1">
+      <x:c r="A16" t="str">
+        <x:v>Demo</x:v>
+      </x:c>
+      <x:c r="B16" t="str">
+        <x:v>SMW001</x:v>
+      </x:c>
+      <x:c r="C16" t="str">
+        <x:v>select_missing_words</x:v>
+      </x:c>
+      <x:c r="D16" t="str">
+        <x:v>SelectMissingWords</x:v>
+      </x:c>
+      <x:c r="E16" s="12" t="str">
+        <x:v>The derivative of $x^2$ is [[1]].</x:v>
+      </x:c>
+      <x:c r="F16"/>
+      <x:c r="G16"/>
+      <x:c r="H16"/>
+      <x:c r="I16"/>
+      <x:c r="J16"/>
+      <x:c r="K16"/>
+      <x:c r="L16"/>
+      <x:c r="M16"/>
+      <x:c r="N16" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="O16" t="str">
+        <x:v>x</x:v>
+      </x:c>
+      <x:c r="P16" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="Q16" t="str">
+        <x:v>FALSE</x:v>
+      </x:c>
+      <x:c r="R16"/>
+      <x:c r="S16"/>
+      <x:c r="T16"/>
+      <x:c r="U16" t="str">
+        <x:v>Đáp án nhiễu.</x:v>
+      </x:c>
+      <x:c r="V16" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="30" customHeight="1">
+      <x:c r="A17" t="str">
+        <x:v>Demo</x:v>
+      </x:c>
+      <x:c r="B17" t="str">
+        <x:v>C002</x:v>
+      </x:c>
+      <x:c r="C17" t="str">
+        <x:v>cloze</x:v>
+      </x:c>
+      <x:c r="D17" t="str">
+        <x:v>Cloze LaTeX</x:v>
+      </x:c>
+      <x:c r="E17" s="12" t="str">
+        <x:v>Tính $\sqrt{16}$ = {1:NUMERICAL:=4:0}.</x:v>
+      </x:c>
+      <x:c r="F17"/>
+      <x:c r="G17"/>
+      <x:c r="H17"/>
+      <x:c r="I17"/>
+      <x:c r="J17"/>
+      <x:c r="K17"/>
+      <x:c r="L17"/>
+      <x:c r="M17"/>
+      <x:c r="N17"/>
+      <x:c r="O17"/>
+      <x:c r="P17"/>
+      <x:c r="Q17"/>
+      <x:c r="R17"/>
+      <x:c r="S17"/>
+      <x:c r="T17"/>
+      <x:c r="U17"/>
+      <x:c r="V17" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:dataValidations count="2">
     <x:dataValidation type="list" sqref="C2:C200">
-      <x:formula1>_Allowed_Values!$A$2:$A$11</x:formula1>
+      <x:formula1>_Allowed_Values!$A$2:$A$12</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="Q2:Q200">
       <x:formula1>_Allowed_Values!$B$2:$B$3</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="18" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="14" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="22" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="24" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="46" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="12" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="12" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="12" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="34" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="10" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="29" t="str">
+        <x:v>category</x:v>
+      </x:c>
+      <x:c r="B1" s="29" t="str">
+        <x:v>question_id</x:v>
+      </x:c>
+      <x:c r="C1" s="29" t="str">
+        <x:v>type</x:v>
+      </x:c>
+      <x:c r="D1" s="29" t="str">
+        <x:v>question_name</x:v>
+      </x:c>
+      <x:c r="E1" s="29" t="str">
+        <x:v>question_text</x:v>
+      </x:c>
+      <x:c r="F1" s="29" t="str">
+        <x:v>drag_no</x:v>
+      </x:c>
+      <x:c r="G1" s="29" t="str">
+        <x:v>drag_text</x:v>
+      </x:c>
+      <x:c r="H1" s="29" t="str">
+        <x:v>group</x:v>
+      </x:c>
+      <x:c r="I1" s="29" t="str">
+        <x:v>explanation</x:v>
+      </x:c>
+      <x:c r="J1" s="29" t="str">
+        <x:v>grade</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="27" t="str">
+        <x:v>Tiếng Anh/Grammar</x:v>
+      </x:c>
+      <x:c r="B2" s="27" t="str">
+        <x:v>SMW001</x:v>
+      </x:c>
+      <x:c r="C2" s="27" t="str">
+        <x:v>select_missing_words</x:v>
+      </x:c>
+      <x:c r="D2" s="27" t="str">
+        <x:v>Select missing words 1</x:v>
+      </x:c>
+      <x:c r="E2" s="27" t="str">
+        <x:v>I [[1]] a student. She [[2]] a teacher.</x:v>
+      </x:c>
+      <x:c r="F2" s="27" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G2" s="27" t="str">
+        <x:v>am</x:v>
+      </x:c>
+      <x:c r="H2" s="27" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I2" s="27" t="str">
+        <x:v>Chọn đúng động từ trong hộp thả xuống.</x:v>
+      </x:c>
+      <x:c r="J2" s="27" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="27" t="str">
+        <x:v>Tiếng Anh/Grammar</x:v>
+      </x:c>
+      <x:c r="B3" s="27" t="str">
+        <x:v>SMW001</x:v>
+      </x:c>
+      <x:c r="C3" s="27" t="str">
+        <x:v>select_missing_words</x:v>
+      </x:c>
+      <x:c r="D3" s="27" t="str">
+        <x:v>Select missing words 1</x:v>
+      </x:c>
+      <x:c r="E3" s="27" t="str">
+        <x:v>I [[1]] a student. She [[2]] a teacher.</x:v>
+      </x:c>
+      <x:c r="F3" s="27" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="G3" s="27" t="str">
+        <x:v>is</x:v>
+      </x:c>
+      <x:c r="H3" s="27" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I3" s="27"/>
+      <x:c r="J3" s="27" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="27" t="str">
+        <x:v>Tiếng Anh/Grammar</x:v>
+      </x:c>
+      <x:c r="B4" s="27" t="str">
+        <x:v>SMW001</x:v>
+      </x:c>
+      <x:c r="C4" s="27" t="str">
+        <x:v>select_missing_words</x:v>
+      </x:c>
+      <x:c r="D4" s="27" t="str">
+        <x:v>Select missing words 1</x:v>
+      </x:c>
+      <x:c r="E4" s="27" t="str">
+        <x:v>I [[1]] a student. She [[2]] a teacher.</x:v>
+      </x:c>
+      <x:c r="F4" s="27" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="G4" s="27" t="str">
+        <x:v>are</x:v>
+      </x:c>
+      <x:c r="H4" s="27" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I4" s="27" t="str">
+        <x:v>Dòng drag_no 3 là lựa chọn nhiễu.</x:v>
+      </x:c>
+      <x:c r="J4" s="27" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:dataValidations count="1">
+    <x:dataValidation type="list" sqref="C2:C200">
+      <x:formula1>_Allowed_Values!$A$2:$A$12</x:formula1>
+    </x:dataValidation>
+  </x:dataValidations>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="1">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ree5a41de31e04f08"/>
+  </x:tableParts>
 </x:worksheet>
 </file>
 
@@ -1346,7 +1727,7 @@
         <x:v>type</x:v>
       </x:c>
       <x:c r="B7" s="12" t="str">
-        <x:v>Dùng một trong các giá trị: single, multi, truefalse, shortanswer, numerical, matching, dragdrop_text, essay, description, cloze.</x:v>
+        <x:v>Dùng một trong các giá trị: single, multi, truefalse, shortanswer, numerical, matching, dragdrop_text, select_missing_words, essay, description, cloze.</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -1383,33 +1764,49 @@
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="12" t="str">
-        <x:v>dragdrop_text</x:v>
+        <x:v>cloze</x:v>
       </x:c>
       <x:c r="B12" s="12" t="str">
-        <x:v>question_text phải chứa [[1]], [[2]], ...; mỗi dòng khai báo drag_no + drag_text. drag_no không có trong text sẽ là đáp án nhiễu.</x:v>
+        <x:v>Nhập cú pháp Embedded answers trực tiếp trong question_text, ví dụ {1:SHORTANSWER:=Hà Nội}. Có thể chứa LaTeX như $x^2$.</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="12" t="str">
-        <x:v>unlimited</x:v>
+        <x:v>dragdrop_text</x:v>
       </x:c>
       <x:c r="B13" s="12" t="str">
-        <x:v>TRUE nếu lựa chọn kéo-thả được dùng lại nhiều lần; FALSE hoặc bỏ trống nếu không.</x:v>
+        <x:v>question_text phải chứa [[1]], [[2]], ...; mỗi dòng khai báo drag_no + drag_text. drag_no không có trong text sẽ là đáp án nhiễu.</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="12" t="str">
-        <x:v>grade</x:v>
+        <x:v>select_missing_words</x:v>
       </x:c>
       <x:c r="B14" s="12" t="str">
-        <x:v>Điểm câu hỏi. Nếu bỏ trống, app mặc định 1; description mặc định 0.</x:v>
+        <x:v>Tương tự dragdrop_text nhưng Moodle hiển thị dạng hộp chọn thả xuống, xuất XML type gapselect.</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="12" t="str">
+        <x:v>unlimited</x:v>
+      </x:c>
+      <x:c r="B15" s="12" t="str">
+        <x:v>TRUE nếu lựa chọn kéo-thả được dùng lại nhiều lần; FALSE hoặc bỏ trống nếu không.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" t="str">
+        <x:v>grade</x:v>
+      </x:c>
+      <x:c r="B16" t="str">
+        <x:v>Điểm câu hỏi. Nếu bỏ trống, app mặc định 1; description mặc định 0.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" t="str">
         <x:v>Import Moodle</x:v>
       </x:c>
-      <x:c r="B15" s="12" t="str">
+      <x:c r="B17" t="str">
         <x:v>Vào Moodle → Question bank → Import → Moodle XML format → chọn file XML app xuất ra.</x:v>
       </x:c>
     </x:row>
@@ -1551,7 +1948,7 @@
   </x:sheetData>
   <x:dataValidations count="2">
     <x:dataValidation type="list" sqref="C2:C200">
-      <x:formula1>_Allowed_Values!$A$2:$A$11</x:formula1>
+      <x:formula1>_Allowed_Values!$A$2:$A$12</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="K2:K200">
       <x:formula1>_Allowed_Values!$C$2:$C$9</x:formula1>
@@ -1693,7 +2090,7 @@
   </x:sheetData>
   <x:dataValidations count="1">
     <x:dataValidation type="list" sqref="C2:C200">
-      <x:formula1>_Allowed_Values!$A$2:$A$11</x:formula1>
+      <x:formula1>_Allowed_Values!$A$2:$A$12</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1789,7 +2186,7 @@
   </x:sheetData>
   <x:dataValidations count="2">
     <x:dataValidation type="list" sqref="C2:C200">
-      <x:formula1>_Allowed_Values!$A$2:$A$11</x:formula1>
+      <x:formula1>_Allowed_Values!$A$2:$A$12</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="F2:F200">
       <x:formula1>_Allowed_Values!$B$2:$B$3</x:formula1>
@@ -1889,7 +2286,7 @@
   </x:sheetData>
   <x:dataValidations count="1">
     <x:dataValidation type="list" sqref="C2:C200">
-      <x:formula1>_Allowed_Values!$A$2:$A$11</x:formula1>
+      <x:formula1>_Allowed_Values!$A$2:$A$12</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1994,7 +2391,7 @@
   </x:sheetData>
   <x:dataValidations count="1">
     <x:dataValidation type="list" sqref="C2:C200">
-      <x:formula1>_Allowed_Values!$A$2:$A$11</x:formula1>
+      <x:formula1>_Allowed_Values!$A$2:$A$12</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2123,7 +2520,7 @@
   </x:sheetData>
   <x:dataValidations count="1">
     <x:dataValidation type="list" sqref="C2:C200">
-      <x:formula1>_Allowed_Values!$A$2:$A$11</x:formula1>
+      <x:formula1>_Allowed_Values!$A$2:$A$12</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2381,7 +2778,7 @@
   </x:sheetData>
   <x:dataValidations count="2">
     <x:dataValidation type="list" sqref="C2:C200">
-      <x:formula1>_Allowed_Values!$A$2:$A$11</x:formula1>
+      <x:formula1>_Allowed_Values!$A$2:$A$12</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="I2:I200">
       <x:formula1>_Allowed_Values!$B$2:$B$3</x:formula1>

</xml_diff>

<commit_message>
feat: add support for cloze question type with validation and rendering enhancements
</commit_message>
<xml_diff>
--- a/public/templates/moodle_xml_sheet_templates.xlsx
+++ b/public/templates/moodle_xml_sheet_templates.xlsx
@@ -2,19 +2,20 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Allowed_Values" sheetId="1" r:id="R8908574161f74c05"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Huong_Dan" sheetId="2" r:id="R756b5b2b5d164d69"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_Single_Choice" sheetId="3" r:id="R09164b6849ea46fa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_Multiple_Choice" sheetId="4" r:id="R4c45caa7cd3b4b63"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_TrueFalse" sheetId="5" r:id="R92014d83ad394f0b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_ShortAnswer" sheetId="6" r:id="R1e7eddc003fc46ef"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_Numerical" sheetId="7" r:id="R729db0cace884da7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_Matching" sheetId="8" r:id="Rb73f3abeb1c94532"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_DragDrop_Text" sheetId="9" r:id="R70b91db75ff949b9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_Essay_Desc_Cloze" sheetId="10" r:id="R2a9cae92b9344d19"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_Reading_Passage" sheetId="11" r:id="Rf064df3fa29a410e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_Full_Demo" sheetId="12" r:id="Rbb757e08f9334aae"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_Select_Missing_Words" sheetId="13" r:id="R1ca4d755589044c4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Allowed_Values" sheetId="1" r:id="R7756809cbfe54a05"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Huong_Dan" sheetId="2" r:id="R85f3e0f3fef24a05"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_Single_Choice" sheetId="3" r:id="R9b4447fd0d7c4663"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_Multiple_Choice" sheetId="4" r:id="R01f2ca4d3b1a4df8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_TrueFalse" sheetId="5" r:id="Red3a006a82904bd5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_ShortAnswer" sheetId="6" r:id="Rcf6b7c0a94854a3c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_Numerical" sheetId="7" r:id="Rd98b74ceb7fb43ed"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_Matching" sheetId="8" r:id="R0938a35aa8064d9f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_DragDrop_Text" sheetId="9" r:id="Rda6f5c902d5c46e1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_Essay_Desc_Cloze" sheetId="10" r:id="R1f55ec477bd843fc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_Reading_Passage" sheetId="11" r:id="R46cd057d8c404de9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_Full_Demo" sheetId="12" r:id="Rfeb44d4ac097466f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_Select_Missing_Words" sheetId="13" r:id="Rfa34d5e4bdb5435d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12_Cloze_Many_In_One" sheetId="14" r:id="Rb7c3f5372c004ace"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -43,7 +44,7 @@
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="7">
+  <x:fills count="12">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -58,6 +59,31 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFDBEAFE"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF2445B6"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF2445B6"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF2445B6"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF2445B6"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF2445B6"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -97,7 +123,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="30">
+  <x:cellXfs count="47">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -162,6 +188,41 @@
     <x:xf numFmtId="0" fontId="1" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="7" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="8" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="9" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="10" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="11" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -182,6 +243,28 @@
     <x:tableColumn id="8" name="group"/>
     <x:tableColumn id="9" name="explanation"/>
     <x:tableColumn id="10" name="grade"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="ClozeTableInput" displayName="ClozeTableInput" ref="A1:N9" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="14">
+    <x:tableColumn id="1" name="category"/>
+    <x:tableColumn id="2" name="question_id"/>
+    <x:tableColumn id="3" name="type"/>
+    <x:tableColumn id="4" name="question_name"/>
+    <x:tableColumn id="5" name="question_text"/>
+    <x:tableColumn id="6" name="cloze_answer_type"/>
+    <x:tableColumn id="7" name="correct_answer"/>
+    <x:tableColumn id="8" name="option_a"/>
+    <x:tableColumn id="9" name="option_b"/>
+    <x:tableColumn id="10" name="option_c"/>
+    <x:tableColumn id="11" name="option_d"/>
+    <x:tableColumn id="12" name="tolerance"/>
+    <x:tableColumn id="13" name="explanation"/>
+    <x:tableColumn id="14" name="grade"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -1672,7 +1755,373 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ree5a41de31e04f08"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8b606b6ce1e94a19"/>
+  </x:tableParts>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="18" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="18" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="10" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="28" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="42" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="18" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="22" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="18" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="18" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="18" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="18" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="12" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="42" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="10" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="46" t="str">
+        <x:v>category</x:v>
+      </x:c>
+      <x:c r="B1" s="46" t="str">
+        <x:v>question_id</x:v>
+      </x:c>
+      <x:c r="C1" s="46" t="str">
+        <x:v>type</x:v>
+      </x:c>
+      <x:c r="D1" s="46" t="str">
+        <x:v>question_name</x:v>
+      </x:c>
+      <x:c r="E1" s="46" t="str">
+        <x:v>question_text</x:v>
+      </x:c>
+      <x:c r="F1" s="46" t="str">
+        <x:v>cloze_answer_type</x:v>
+      </x:c>
+      <x:c r="G1" s="46" t="str">
+        <x:v>correct_answer</x:v>
+      </x:c>
+      <x:c r="H1" s="46" t="str">
+        <x:v>option_a</x:v>
+      </x:c>
+      <x:c r="I1" s="46" t="str">
+        <x:v>option_b</x:v>
+      </x:c>
+      <x:c r="J1" s="46" t="str">
+        <x:v>option_c</x:v>
+      </x:c>
+      <x:c r="K1" s="46" t="str">
+        <x:v>option_d</x:v>
+      </x:c>
+      <x:c r="L1" s="46" t="str">
+        <x:v>tolerance</x:v>
+      </x:c>
+      <x:c r="M1" s="46" t="str">
+        <x:v>explanation</x:v>
+      </x:c>
+      <x:c r="N1" s="46" t="str">
+        <x:v>grade</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="46" customHeight="1">
+      <x:c r="A2" s="27" t="str">
+        <x:v>Demo/Cloze</x:v>
+      </x:c>
+      <x:c r="B2" s="27" t="str">
+        <x:v>CLZ_TABLE_001</x:v>
+      </x:c>
+      <x:c r="C2" s="27" t="str">
+        <x:v>cloze</x:v>
+      </x:c>
+      <x:c r="D2" s="27" t="str">
+        <x:v>Một câu Cloze nhập từng dòng</x:v>
+      </x:c>
+      <x:c r="E2" s="27" t="str">
+        <x:v>Thủ đô Việt Nam là gì?</x:v>
+      </x:c>
+      <x:c r="F2" s="27" t="str">
+        <x:v>shortanswer</x:v>
+      </x:c>
+      <x:c r="G2" s="27" t="str">
+        <x:v>Hà Nội;Ha Noi</x:v>
+      </x:c>
+      <x:c r="H2" s="27" t="str"/>
+      <x:c r="I2" s="27" t="str"/>
+      <x:c r="J2" s="27" t="str"/>
+      <x:c r="K2" s="27" t="str"/>
+      <x:c r="L2" s="27" t="str"/>
+      <x:c r="M2" s="27" t="str">
+        <x:v>Sinh SHORTANSWER.</x:v>
+      </x:c>
+      <x:c r="N2" s="27" t="n">
+        <x:v>7</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="46" customHeight="1">
+      <x:c r="A3" s="27" t="str">
+        <x:v>Demo/Cloze</x:v>
+      </x:c>
+      <x:c r="B3" s="27" t="str">
+        <x:v>CLZ_TABLE_001</x:v>
+      </x:c>
+      <x:c r="C3" s="27" t="str">
+        <x:v>cloze</x:v>
+      </x:c>
+      <x:c r="D3" s="27" t="str">
+        <x:v>Một câu Cloze nhập từng dòng</x:v>
+      </x:c>
+      <x:c r="E3" s="27" t="str">
+        <x:v>Viết moodle bằng chữ HOA.</x:v>
+      </x:c>
+      <x:c r="F3" s="27" t="str">
+        <x:v>shortanswer_c</x:v>
+      </x:c>
+      <x:c r="G3" s="27" t="str">
+        <x:v>MOODLE</x:v>
+      </x:c>
+      <x:c r="H3" s="27" t="str"/>
+      <x:c r="I3" s="27" t="str"/>
+      <x:c r="J3" s="27" t="str"/>
+      <x:c r="K3" s="27" t="str"/>
+      <x:c r="L3" s="27" t="str"/>
+      <x:c r="M3" s="27" t="str">
+        <x:v>Sinh SHORTANSWER_C, phân biệt hoa/thường.</x:v>
+      </x:c>
+      <x:c r="N3" s="27" t="str"/>
+    </x:row>
+    <x:row r="4" ht="46" customHeight="1">
+      <x:c r="A4" s="27" t="str">
+        <x:v>Demo/Cloze</x:v>
+      </x:c>
+      <x:c r="B4" s="27" t="str">
+        <x:v>CLZ_TABLE_001</x:v>
+      </x:c>
+      <x:c r="C4" s="27" t="str">
+        <x:v>cloze</x:v>
+      </x:c>
+      <x:c r="D4" s="27" t="str">
+        <x:v>Một câu Cloze nhập từng dòng</x:v>
+      </x:c>
+      <x:c r="E4" s="27" t="str">
+        <x:v>2 + 3 bằng bao nhiêu?</x:v>
+      </x:c>
+      <x:c r="F4" s="27" t="str">
+        <x:v>numerical</x:v>
+      </x:c>
+      <x:c r="G4" s="27" t="str">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="H4" s="27" t="str"/>
+      <x:c r="I4" s="27" t="str"/>
+      <x:c r="J4" s="27" t="str"/>
+      <x:c r="K4" s="27" t="str"/>
+      <x:c r="L4" s="27" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M4" s="27" t="str">
+        <x:v>Sinh NUMERICAL.</x:v>
+      </x:c>
+      <x:c r="N4" s="27" t="str"/>
+    </x:row>
+    <x:row r="5" ht="46" customHeight="1">
+      <x:c r="A5" s="27" t="str">
+        <x:v>Demo/Cloze</x:v>
+      </x:c>
+      <x:c r="B5" s="27" t="str">
+        <x:v>CLZ_TABLE_001</x:v>
+      </x:c>
+      <x:c r="C5" s="27" t="str">
+        <x:v>cloze</x:v>
+      </x:c>
+      <x:c r="D5" s="27" t="str">
+        <x:v>Một câu Cloze nhập từng dòng</x:v>
+      </x:c>
+      <x:c r="E5" s="27" t="str">
+        <x:v>Số 7 thuộc loại nào?</x:v>
+      </x:c>
+      <x:c r="F5" s="27" t="str">
+        <x:v>multichoice</x:v>
+      </x:c>
+      <x:c r="G5" s="27" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="H5" s="27" t="str">
+        <x:v>số nguyên tố</x:v>
+      </x:c>
+      <x:c r="I5" s="27" t="str">
+        <x:v>số chẵn</x:v>
+      </x:c>
+      <x:c r="J5" s="27" t="str">
+        <x:v>số âm</x:v>
+      </x:c>
+      <x:c r="K5" s="27" t="str">
+        <x:v>hợp số</x:v>
+      </x:c>
+      <x:c r="L5" s="27" t="str"/>
+      <x:c r="M5" s="27" t="str">
+        <x:v>Sinh MULTICHOICE dạng dropdown.</x:v>
+      </x:c>
+      <x:c r="N5" s="27" t="str"/>
+    </x:row>
+    <x:row r="6" ht="46" customHeight="1">
+      <x:c r="A6" s="27" t="str">
+        <x:v>Demo/Cloze</x:v>
+      </x:c>
+      <x:c r="B6" s="27" t="str">
+        <x:v>CLZ_TABLE_001</x:v>
+      </x:c>
+      <x:c r="C6" s="27" t="str">
+        <x:v>cloze</x:v>
+      </x:c>
+      <x:c r="D6" s="27" t="str">
+        <x:v>Một câu Cloze nhập từng dòng</x:v>
+      </x:c>
+      <x:c r="E6" s="27" t="str">
+        <x:v>Chọn đáp án hiển thị dọc.</x:v>
+      </x:c>
+      <x:c r="F6" s="27" t="str">
+        <x:v>mcv</x:v>
+      </x:c>
+      <x:c r="G6" s="27" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="H6" s="27" t="str">
+        <x:v>1. Sai</x:v>
+      </x:c>
+      <x:c r="I6" s="27" t="str">
+        <x:v>2. Cũng sai</x:v>
+      </x:c>
+      <x:c r="J6" s="27" t="str">
+        <x:v>3. Đúng</x:v>
+      </x:c>
+      <x:c r="K6" s="27" t="str">
+        <x:v>4. Nửa đúng</x:v>
+      </x:c>
+      <x:c r="L6" s="27" t="str"/>
+      <x:c r="M6" s="27" t="str">
+        <x:v>Sinh MCV, Moodle hiển thị lựa chọn dạng dọc.</x:v>
+      </x:c>
+      <x:c r="N6" s="27" t="str"/>
+    </x:row>
+    <x:row r="7" ht="46" customHeight="1">
+      <x:c r="A7" s="27" t="str">
+        <x:v>Demo/Cloze</x:v>
+      </x:c>
+      <x:c r="B7" s="27" t="str">
+        <x:v>CLZ_TABLE_001</x:v>
+      </x:c>
+      <x:c r="C7" s="27" t="str">
+        <x:v>cloze</x:v>
+      </x:c>
+      <x:c r="D7" s="27" t="str">
+        <x:v>Một câu Cloze nhập từng dòng</x:v>
+      </x:c>
+      <x:c r="E7" s="27" t="str">
+        <x:v>Chọn đáp án hiển thị ngang.</x:v>
+      </x:c>
+      <x:c r="F7" s="27" t="str">
+        <x:v>mch</x:v>
+      </x:c>
+      <x:c r="G7" s="27" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="H7" s="27" t="str">
+        <x:v>a. Sai</x:v>
+      </x:c>
+      <x:c r="I7" s="27" t="str">
+        <x:v>b. Cũng sai</x:v>
+      </x:c>
+      <x:c r="J7" s="27" t="str">
+        <x:v>c. Đúng</x:v>
+      </x:c>
+      <x:c r="K7" s="27" t="str">
+        <x:v>d. Nửa đúng</x:v>
+      </x:c>
+      <x:c r="L7" s="27" t="str"/>
+      <x:c r="M7" s="27" t="str">
+        <x:v>Sinh MCH, Moodle hiển thị lựa chọn dạng ngang.</x:v>
+      </x:c>
+      <x:c r="N7" s="27" t="str"/>
+    </x:row>
+    <x:row r="8" ht="46" customHeight="1">
+      <x:c r="A8" s="27" t="str">
+        <x:v>Demo/Cloze</x:v>
+      </x:c>
+      <x:c r="B8" s="27" t="str">
+        <x:v>CLZ_TABLE_001</x:v>
+      </x:c>
+      <x:c r="C8" s="27" t="str">
+        <x:v>cloze</x:v>
+      </x:c>
+      <x:c r="D8" s="27" t="str">
+        <x:v>Một câu Cloze nhập từng dòng</x:v>
+      </x:c>
+      <x:c r="E8" s="27" t="str">
+        <x:v>Với công thức \(S=\pi r^2\), hằng số cần điền là gì?</x:v>
+      </x:c>
+      <x:c r="F8" s="27" t="str">
+        <x:v>shortanswer</x:v>
+      </x:c>
+      <x:c r="G8" s="27" t="str">
+        <x:v>pi</x:v>
+      </x:c>
+      <x:c r="H8" s="27" t="str"/>
+      <x:c r="I8" s="27" t="str"/>
+      <x:c r="J8" s="27" t="str"/>
+      <x:c r="K8" s="27" t="str"/>
+      <x:c r="L8" s="27" t="str"/>
+      <x:c r="M8" s="27" t="str">
+        <x:v>Có thể viết LaTeX trong question_text.</x:v>
+      </x:c>
+      <x:c r="N8" s="27" t="str"/>
+    </x:row>
+    <x:row r="9" ht="46" customHeight="1">
+      <x:c r="A9" s="27" t="str">
+        <x:v>Demo/Cloze</x:v>
+      </x:c>
+      <x:c r="B9" s="27" t="str">
+        <x:v>CLZ_TABLE_002</x:v>
+      </x:c>
+      <x:c r="C9" s="27" t="str">
+        <x:v>cloze</x:v>
+      </x:c>
+      <x:c r="D9" s="27" t="str">
+        <x:v>Một câu Cloze khác</x:v>
+      </x:c>
+      <x:c r="E9" s="27" t="str">
+        <x:v>The capital of Vietnam is [[answer]].</x:v>
+      </x:c>
+      <x:c r="F9" s="27" t="str">
+        <x:v>shortanswer</x:v>
+      </x:c>
+      <x:c r="G9" s="27" t="str">
+        <x:v>Hanoi;Ha Noi</x:v>
+      </x:c>
+      <x:c r="H9" s="27" t="str"/>
+      <x:c r="I9" s="27" t="str"/>
+      <x:c r="J9" s="27" t="str"/>
+      <x:c r="K9" s="27" t="str"/>
+      <x:c r="L9" s="27" t="str"/>
+      <x:c r="M9" s="27" t="str">
+        <x:v>Có thể đặt [[answer]] để app chèn ô trả lời đúng vị trí.</x:v>
+      </x:c>
+      <x:c r="N9" s="27" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:dataValidations count="2">
+    <x:dataValidation type="list" sqref="C2:C200">
+      <x:formula1>_Allowed_Values!$A$2:$A$12</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="F2:F200">
+      <x:formula1>"shortanswer,shortanswer_c,numerical,multichoice,mcv,mch"</x:formula1>
+    </x:dataValidation>
+  </x:dataValidations>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="1">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re2187623a8044b88"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1767,7 +2216,7 @@
         <x:v>cloze</x:v>
       </x:c>
       <x:c r="B12" s="12" t="str">
-        <x:v>Nhập cú pháp Embedded answers trực tiếp trong question_text, ví dụ {1:SHORTANSWER:=Hà Nội}. Có thể chứa LaTeX như $x^2$.</x:v>
+        <x:v>Có thể nhập sẵn cú pháp Embedded answers trong question_text, hoặc nhập dạng bảng nhiều dòng cùng question_id. cloze_answer_type hỗ trợ: shortanswer, shortanswer_c, numerical, multichoice, mcv, mch. App sẽ tự sinh mã SHORTANSWER/SHORTANSWER_C/NUMERICAL/MULTICHOICE/MCV/MCH.</x:v>
       </x:c>
     </x:row>
     <x:row r="13">

</xml_diff>

<commit_message>
feat: add shuffle answers and show correct when wrong options to question types
</commit_message>
<xml_diff>
--- a/public/templates/moodle_xml_sheet_templates.xlsx
+++ b/public/templates/moodle_xml_sheet_templates.xlsx
@@ -2,20 +2,20 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Allowed_Values" sheetId="1" r:id="R7756809cbfe54a05"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Huong_Dan" sheetId="2" r:id="R85f3e0f3fef24a05"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_Single_Choice" sheetId="3" r:id="R9b4447fd0d7c4663"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_Multiple_Choice" sheetId="4" r:id="R01f2ca4d3b1a4df8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_TrueFalse" sheetId="5" r:id="Red3a006a82904bd5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_ShortAnswer" sheetId="6" r:id="Rcf6b7c0a94854a3c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_Numerical" sheetId="7" r:id="Rd98b74ceb7fb43ed"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_Matching" sheetId="8" r:id="R0938a35aa8064d9f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_DragDrop_Text" sheetId="9" r:id="Rda6f5c902d5c46e1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_Essay_Desc_Cloze" sheetId="10" r:id="R1f55ec477bd843fc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_Reading_Passage" sheetId="11" r:id="R46cd057d8c404de9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_Full_Demo" sheetId="12" r:id="Rfeb44d4ac097466f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_Select_Missing_Words" sheetId="13" r:id="Rfa34d5e4bdb5435d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12_Cloze_Many_In_One" sheetId="14" r:id="Rb7c3f5372c004ace"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Allowed_Values" sheetId="1" r:id="Rcec0a542981e40d0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Huong_Dan" sheetId="2" r:id="R62aa9b46b6ae4da6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_Single_Choice" sheetId="3" r:id="R436118ae4f1f48fc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_Multiple_Choice" sheetId="4" r:id="Rd6742cd6601e47ac"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_TrueFalse" sheetId="5" r:id="R0d789be7aec04d22"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_ShortAnswer" sheetId="6" r:id="R3ab26ada3ee14149"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_Numerical" sheetId="7" r:id="Radf0e633a977447f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_Matching" sheetId="8" r:id="Rfbcc500d38a346c1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_DragDrop_Text" sheetId="9" r:id="Rae573c0837774eca"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_Essay_Desc_Cloze" sheetId="10" r:id="R3401de5ebee54700"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_Reading_Passage" sheetId="11" r:id="Rdda0ec4411314db2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_Full_Demo" sheetId="12" r:id="Rf27e5f82d7854367"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_Select_Missing_Words" sheetId="13" r:id="R2b1fb838d15b40b6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12_Cloze_Many_In_One" sheetId="14" r:id="R468f589aa0de43b8"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -26,7 +26,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:fonts count="3">
+  <x:fonts count="4">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -43,8 +43,13 @@
       <x:color rgb="FF0F172A"/>
       <x:name val="Carlito"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:name val="Carlito"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="12">
+  <x:fills count="15">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -101,6 +106,21 @@
         <x:fgColor rgb="FF2445B6"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF2445B6"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F4E78"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE2F0D9"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="3">
     <x:border/>
@@ -123,7 +143,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="47">
+  <x:cellXfs count="58">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -223,6 +243,31 @@
     <x:xf numFmtId="0" fontId="1" fillId="11" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="12" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="13" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="14" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -249,22 +294,24 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="ClozeTableInput" displayName="ClozeTableInput" ref="A1:N9" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:tableColumns count="14">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="ClozeTableInput" displayName="ClozeTableInput" ref="A1:P9" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="16">
     <x:tableColumn id="1" name="category"/>
     <x:tableColumn id="2" name="question_id"/>
     <x:tableColumn id="3" name="type"/>
     <x:tableColumn id="4" name="question_name"/>
-    <x:tableColumn id="5" name="question_text"/>
-    <x:tableColumn id="6" name="cloze_answer_type"/>
-    <x:tableColumn id="7" name="correct_answer"/>
-    <x:tableColumn id="8" name="option_a"/>
-    <x:tableColumn id="9" name="option_b"/>
-    <x:tableColumn id="10" name="option_c"/>
-    <x:tableColumn id="11" name="option_d"/>
-    <x:tableColumn id="12" name="tolerance"/>
-    <x:tableColumn id="13" name="explanation"/>
-    <x:tableColumn id="14" name="grade"/>
+    <x:tableColumn id="5" name="passage_id"/>
+    <x:tableColumn id="6" name="passage_text"/>
+    <x:tableColumn id="7" name="question_text"/>
+    <x:tableColumn id="8" name="cloze_answer_type"/>
+    <x:tableColumn id="9" name="correct_answer"/>
+    <x:tableColumn id="10" name="option_a"/>
+    <x:tableColumn id="11" name="option_b"/>
+    <x:tableColumn id="12" name="option_c"/>
+    <x:tableColumn id="13" name="option_d"/>
+    <x:tableColumn id="14" name="tolerance"/>
+    <x:tableColumn id="15" name="explanation"/>
+    <x:tableColumn id="16" name="grade"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -1755,7 +1802,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8b606b6ce1e94a19"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6d8d32c9c6434114"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1768,315 +1815,406 @@
     <x:col min="2" max="2" width="18" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="10" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="28" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="42" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="18" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="22" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="14" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="52" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="38" hidden="0" customWidth="1"/>
     <x:col min="8" max="8" width="18" hidden="0" customWidth="1"/>
     <x:col min="9" max="9" width="18" hidden="0" customWidth="1"/>
     <x:col min="10" max="10" width="18" hidden="0" customWidth="1"/>
-    <x:col min="11" max="11" width="18" hidden="0" customWidth="1"/>
-    <x:col min="12" max="12" width="12" hidden="0" customWidth="1"/>
-    <x:col min="13" max="13" width="42" hidden="0" customWidth="1"/>
-    <x:col min="14" max="14" width="10" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="30" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="30" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="30" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="30" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="30" hidden="0" customWidth="1"/>
+    <x:col min="16" max="16" width="10" hidden="0" customWidth="1"/>
+    <x:col min="17" max="17" width="42" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
-      <x:c r="A1" s="46" t="str">
+      <x:c r="A1" s="51" t="str">
         <x:v>category</x:v>
       </x:c>
-      <x:c r="B1" s="46" t="str">
+      <x:c r="B1" s="51" t="str">
         <x:v>question_id</x:v>
       </x:c>
-      <x:c r="C1" s="46" t="str">
+      <x:c r="C1" s="51" t="str">
         <x:v>type</x:v>
       </x:c>
-      <x:c r="D1" s="46" t="str">
+      <x:c r="D1" s="51" t="str">
         <x:v>question_name</x:v>
       </x:c>
-      <x:c r="E1" s="46" t="str">
+      <x:c r="E1" s="51" t="str">
+        <x:v>passage_id</x:v>
+      </x:c>
+      <x:c r="F1" s="51" t="str">
+        <x:v>passage_text</x:v>
+      </x:c>
+      <x:c r="G1" s="51" t="str">
         <x:v>question_text</x:v>
       </x:c>
-      <x:c r="F1" s="46" t="str">
+      <x:c r="H1" s="51" t="str">
         <x:v>cloze_answer_type</x:v>
       </x:c>
-      <x:c r="G1" s="46" t="str">
+      <x:c r="I1" s="51" t="str">
+        <x:v>shuffle_answers</x:v>
+      </x:c>
+      <x:c r="J1" s="51" t="str">
+        <x:v>show_correct_when_wrong</x:v>
+      </x:c>
+      <x:c r="K1" s="51" t="str">
         <x:v>correct_answer</x:v>
       </x:c>
-      <x:c r="H1" s="46" t="str">
+      <x:c r="L1" s="51" t="str">
         <x:v>option_a</x:v>
       </x:c>
-      <x:c r="I1" s="46" t="str">
+      <x:c r="M1" s="51" t="str">
         <x:v>option_b</x:v>
       </x:c>
-      <x:c r="J1" s="46" t="str">
+      <x:c r="N1" s="51" t="str">
         <x:v>option_c</x:v>
       </x:c>
-      <x:c r="K1" s="46" t="str">
+      <x:c r="O1" s="51" t="str">
         <x:v>option_d</x:v>
       </x:c>
-      <x:c r="L1" s="46" t="str">
+      <x:c r="P1" s="51" t="str">
         <x:v>tolerance</x:v>
       </x:c>
-      <x:c r="M1" s="46" t="str">
+      <x:c r="Q1" s="51" t="str">
         <x:v>explanation</x:v>
       </x:c>
-      <x:c r="N1" s="46" t="str">
+      <x:c r="R1" s="51" t="str">
         <x:v>grade</x:v>
       </x:c>
     </x:row>
-    <x:row r="2" ht="46" customHeight="1">
+    <x:row r="2" ht="124" customHeight="1">
       <x:c r="A2" s="27" t="str">
         <x:v>Demo/Cloze</x:v>
       </x:c>
       <x:c r="B2" s="27" t="str">
-        <x:v>CLZ_TABLE_001</x:v>
+        <x:v>CLZ_READING_001</x:v>
       </x:c>
       <x:c r="C2" s="27" t="str">
         <x:v>cloze</x:v>
       </x:c>
       <x:c r="D2" s="27" t="str">
-        <x:v>Một câu Cloze nhập từng dòng</x:v>
+        <x:v>Cloze đọc hiểu có đoạn văn</x:v>
       </x:c>
       <x:c r="E2" s="27" t="str">
-        <x:v>Thủ đô Việt Nam là gì?</x:v>
+        <x:v>NC001</x:v>
       </x:c>
       <x:c r="F2" s="27" t="str">
-        <x:v>shortanswer</x:v>
+        <x:v>Nhà văn Nam Cao (1917-1951) là một trong những nhà văn hiện thực xuất sắc nhất của văn học Việt Nam thế kỷ XX. Ông đặc biệt thành công khi viết về người nông dân và trí thức nghèo. Tác phẩm Chí Phèo không chỉ là câu chuyện về một người nông dân bị tha hóa mà còn là bức tranh hiện thực về xã hội nông thôn Việt Nam trước Cách mạng. Qua nhân vật Chí Phèo, Nam Cao đã đặt ra câu hỏi: ai đã đẩy Chí Phèo vào con đường lưu manh hóa? Đó không chỉ là số phận của một người mà là số phận của cả một tầng lớp trong xã hội cũ. Dù sự nghiệp sáng tác không dài, nhưng những tác phẩm của Nam Cao vẫn giữ nguyên giá trị cho đến ngày nay.</x:v>
       </x:c>
       <x:c r="G2" s="27" t="str">
-        <x:v>Hà Nội;Ha Noi</x:v>
-      </x:c>
-      <x:c r="H2" s="27" t="str"/>
-      <x:c r="I2" s="27" t="str"/>
-      <x:c r="J2" s="27" t="str"/>
-      <x:c r="K2" s="27" t="str"/>
-      <x:c r="L2" s="27" t="str"/>
+        <x:v>Nam Cao sinh năm nào?</x:v>
+      </x:c>
+      <x:c r="H2" s="27" t="str">
+        <x:v>mcv</x:v>
+      </x:c>
+      <x:c r="I2" s="27" t="str">
+        <x:v>TRUE</x:v>
+      </x:c>
+      <x:c r="J2" s="27" t="str">
+        <x:v>TRUE</x:v>
+      </x:c>
+      <x:c r="K2" s="27" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="L2" s="27" t="str">
+        <x:v>1915</x:v>
+      </x:c>
       <x:c r="M2" s="27" t="str">
-        <x:v>Sinh SHORTANSWER.</x:v>
-      </x:c>
-      <x:c r="N2" s="27" t="n">
+        <x:v>1917</x:v>
+      </x:c>
+      <x:c r="N2" s="27" t="str">
+        <x:v>1919</x:v>
+      </x:c>
+      <x:c r="O2" s="27" t="str">
+        <x:v>1921</x:v>
+      </x:c>
+      <x:c r="P2" s="27" t="str"/>
+      <x:c r="Q2" s="27" t="str">
+        <x:v>Nếu chọn sai, Moodle sẽ hiện đáp án đúng cho riêng câu nhỏ này.</x:v>
+      </x:c>
+      <x:c r="R2" s="27" t="n">
         <x:v>7</x:v>
       </x:c>
     </x:row>
-    <x:row r="3" ht="46" customHeight="1">
+    <x:row r="3" ht="54" customHeight="1">
       <x:c r="A3" s="27" t="str">
         <x:v>Demo/Cloze</x:v>
       </x:c>
       <x:c r="B3" s="27" t="str">
-        <x:v>CLZ_TABLE_001</x:v>
+        <x:v>CLZ_READING_001</x:v>
       </x:c>
       <x:c r="C3" s="27" t="str">
         <x:v>cloze</x:v>
       </x:c>
       <x:c r="D3" s="27" t="str">
-        <x:v>Một câu Cloze nhập từng dòng</x:v>
+        <x:v>Cloze đọc hiểu có đoạn văn</x:v>
       </x:c>
       <x:c r="E3" s="27" t="str">
-        <x:v>Viết moodle bằng chữ HOA.</x:v>
-      </x:c>
-      <x:c r="F3" s="27" t="str">
-        <x:v>shortanswer_c</x:v>
-      </x:c>
+        <x:v>NC001</x:v>
+      </x:c>
+      <x:c r="F3" s="27" t="str"/>
       <x:c r="G3" s="27" t="str">
-        <x:v>MOODLE</x:v>
-      </x:c>
-      <x:c r="H3" s="27" t="str"/>
-      <x:c r="I3" s="27" t="str"/>
-      <x:c r="J3" s="27" t="str"/>
-      <x:c r="K3" s="27" t="str"/>
-      <x:c r="L3" s="27" t="str"/>
+        <x:v>Ý chính của đoạn văn là gì?</x:v>
+      </x:c>
+      <x:c r="H3" s="27" t="str">
+        <x:v>mcv</x:v>
+      </x:c>
+      <x:c r="I3" s="27" t="str">
+        <x:v>TRUE</x:v>
+      </x:c>
+      <x:c r="J3" s="27" t="str">
+        <x:v>TRUE</x:v>
+      </x:c>
+      <x:c r="K3" s="27" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="L3" s="27" t="str">
+        <x:v>Nam Cao là nhà văn hiện thực xuất sắc với những tác phẩm có giá trị</x:v>
+      </x:c>
       <x:c r="M3" s="27" t="str">
-        <x:v>Sinh SHORTANSWER_C, phân biệt hoa/thường.</x:v>
-      </x:c>
-      <x:c r="N3" s="27" t="str"/>
-    </x:row>
-    <x:row r="4" ht="46" customHeight="1">
+        <x:v>Chí Phèo là tác phẩm nổi tiếng nhất của Nam Cao</x:v>
+      </x:c>
+      <x:c r="N3" s="27" t="str">
+        <x:v>Nam Cao viết về người nông dân</x:v>
+      </x:c>
+      <x:c r="O3" s="27" t="str">
+        <x:v>Sự nghiệp sáng tác của Nam Cao không dài</x:v>
+      </x:c>
+      <x:c r="P3" s="27" t="str"/>
+      <x:c r="Q3" s="27" t="str"/>
+      <x:c r="R3" s="27" t="str"/>
+    </x:row>
+    <x:row r="4" ht="54" customHeight="1">
       <x:c r="A4" s="27" t="str">
         <x:v>Demo/Cloze</x:v>
       </x:c>
       <x:c r="B4" s="27" t="str">
-        <x:v>CLZ_TABLE_001</x:v>
+        <x:v>CLZ_READING_001</x:v>
       </x:c>
       <x:c r="C4" s="27" t="str">
         <x:v>cloze</x:v>
       </x:c>
       <x:c r="D4" s="27" t="str">
-        <x:v>Một câu Cloze nhập từng dòng</x:v>
+        <x:v>Cloze đọc hiểu có đoạn văn</x:v>
       </x:c>
       <x:c r="E4" s="27" t="str">
-        <x:v>2 + 3 bằng bao nhiêu?</x:v>
-      </x:c>
-      <x:c r="F4" s="27" t="str">
-        <x:v>numerical</x:v>
-      </x:c>
+        <x:v>NC001</x:v>
+      </x:c>
+      <x:c r="F4" s="27" t="str"/>
       <x:c r="G4" s="27" t="str">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="H4" s="27" t="str"/>
-      <x:c r="I4" s="27" t="str"/>
-      <x:c r="J4" s="27" t="str"/>
-      <x:c r="K4" s="27" t="str"/>
+        <x:v>Điều gì có thể suy ra từ đoạn văn?</x:v>
+      </x:c>
+      <x:c r="H4" s="27" t="str">
+        <x:v>mcv</x:v>
+      </x:c>
+      <x:c r="I4" s="27" t="str">
+        <x:v>TRUE</x:v>
+      </x:c>
+      <x:c r="J4" s="27" t="str">
+        <x:v>TRUE</x:v>
+      </x:c>
+      <x:c r="K4" s="27" t="str">
+        <x:v>B</x:v>
+      </x:c>
       <x:c r="L4" s="27" t="str">
-        <x:v>0</x:v>
+        <x:v>Nam Cao chỉ viết về người nông dân</x:v>
       </x:c>
       <x:c r="M4" s="27" t="str">
-        <x:v>Sinh NUMERICAL.</x:v>
-      </x:c>
-      <x:c r="N4" s="27" t="str"/>
-    </x:row>
-    <x:row r="5" ht="46" customHeight="1">
+        <x:v>Nam Cao quan tâm đến số phận người nông dân trong xã hội cũ</x:v>
+      </x:c>
+      <x:c r="N4" s="27" t="str">
+        <x:v>Nam Cao là nhà văn duy nhất viết về nông dân</x:v>
+      </x:c>
+      <x:c r="O4" s="27" t="str">
+        <x:v>Các tác phẩm của Nam Cao đã mất giá trị</x:v>
+      </x:c>
+      <x:c r="P4" s="27" t="str"/>
+      <x:c r="Q4" s="27" t="str"/>
+      <x:c r="R4" s="27" t="str"/>
+    </x:row>
+    <x:row r="5" ht="54" customHeight="1">
       <x:c r="A5" s="27" t="str">
         <x:v>Demo/Cloze</x:v>
       </x:c>
       <x:c r="B5" s="27" t="str">
-        <x:v>CLZ_TABLE_001</x:v>
+        <x:v>CLZ_READING_001</x:v>
       </x:c>
       <x:c r="C5" s="27" t="str">
         <x:v>cloze</x:v>
       </x:c>
       <x:c r="D5" s="27" t="str">
-        <x:v>Một câu Cloze nhập từng dòng</x:v>
+        <x:v>Cloze đọc hiểu có đoạn văn</x:v>
       </x:c>
       <x:c r="E5" s="27" t="str">
-        <x:v>Số 7 thuộc loại nào?</x:v>
-      </x:c>
-      <x:c r="F5" s="27" t="str">
-        <x:v>multichoice</x:v>
-      </x:c>
+        <x:v>NC001</x:v>
+      </x:c>
+      <x:c r="F5" s="27" t="str"/>
       <x:c r="G5" s="27" t="str">
+        <x:v>Từ tha hóa trong đoạn văn có nghĩa gần nhất với từ nào?</x:v>
+      </x:c>
+      <x:c r="H5" s="27" t="str">
+        <x:v>mcv</x:v>
+      </x:c>
+      <x:c r="I5" s="27" t="str">
+        <x:v>TRUE</x:v>
+      </x:c>
+      <x:c r="J5" s="27" t="str">
+        <x:v>TRUE</x:v>
+      </x:c>
+      <x:c r="K5" s="27" t="str">
         <x:v>A</x:v>
       </x:c>
-      <x:c r="H5" s="27" t="str">
-        <x:v>số nguyên tố</x:v>
-      </x:c>
-      <x:c r="I5" s="27" t="str">
-        <x:v>số chẵn</x:v>
-      </x:c>
-      <x:c r="J5" s="27" t="str">
-        <x:v>số âm</x:v>
-      </x:c>
-      <x:c r="K5" s="27" t="str">
-        <x:v>hợp số</x:v>
-      </x:c>
-      <x:c r="L5" s="27" t="str"/>
+      <x:c r="L5" s="27" t="str">
+        <x:v>Suy thoái nhân phẩm</x:v>
+      </x:c>
       <x:c r="M5" s="27" t="str">
-        <x:v>Sinh MULTICHOICE dạng dropdown.</x:v>
-      </x:c>
-      <x:c r="N5" s="27" t="str"/>
-    </x:row>
-    <x:row r="6" ht="46" customHeight="1">
+        <x:v>Trở nên giàu có</x:v>
+      </x:c>
+      <x:c r="N5" s="27" t="str">
+        <x:v>Bị bệnh tật</x:v>
+      </x:c>
+      <x:c r="O5" s="27" t="str">
+        <x:v>Mất nhà cửa</x:v>
+      </x:c>
+      <x:c r="P5" s="27" t="str"/>
+      <x:c r="Q5" s="27" t="str"/>
+      <x:c r="R5" s="27" t="str"/>
+    </x:row>
+    <x:row r="6" ht="54" customHeight="1">
       <x:c r="A6" s="27" t="str">
         <x:v>Demo/Cloze</x:v>
       </x:c>
       <x:c r="B6" s="27" t="str">
-        <x:v>CLZ_TABLE_001</x:v>
+        <x:v>CLZ_READING_001</x:v>
       </x:c>
       <x:c r="C6" s="27" t="str">
         <x:v>cloze</x:v>
       </x:c>
       <x:c r="D6" s="27" t="str">
-        <x:v>Một câu Cloze nhập từng dòng</x:v>
+        <x:v>Cloze đọc hiểu có đoạn văn</x:v>
       </x:c>
       <x:c r="E6" s="27" t="str">
-        <x:v>Chọn đáp án hiển thị dọc.</x:v>
-      </x:c>
-      <x:c r="F6" s="27" t="str">
+        <x:v>NC001</x:v>
+      </x:c>
+      <x:c r="F6" s="27" t="str"/>
+      <x:c r="G6" s="27" t="str">
+        <x:v>Câu Đó không chỉ là số phận của một người mà là số phận của cả một tầng lớp trong xã hội cũ có ý nghĩa gì?</x:v>
+      </x:c>
+      <x:c r="H6" s="27" t="str">
         <x:v>mcv</x:v>
       </x:c>
-      <x:c r="G6" s="27" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="H6" s="27" t="str">
-        <x:v>1. Sai</x:v>
-      </x:c>
       <x:c r="I6" s="27" t="str">
-        <x:v>2. Cũng sai</x:v>
+        <x:v>TRUE</x:v>
       </x:c>
       <x:c r="J6" s="27" t="str">
-        <x:v>3. Đúng</x:v>
+        <x:v>TRUE</x:v>
       </x:c>
       <x:c r="K6" s="27" t="str">
-        <x:v>4. Nửa đúng</x:v>
-      </x:c>
-      <x:c r="L6" s="27" t="str"/>
+        <x:v>D</x:v>
+      </x:c>
+      <x:c r="L6" s="27" t="str">
+        <x:v>Chí Phèo đại diện cho số phận của nhiều người trong xã hội cũ</x:v>
+      </x:c>
       <x:c r="M6" s="27" t="str">
-        <x:v>Sinh MCV, Moodle hiển thị lựa chọn dạng dọc.</x:v>
-      </x:c>
-      <x:c r="N6" s="27" t="str"/>
-    </x:row>
-    <x:row r="7" ht="46" customHeight="1">
+        <x:v>Chỉ có Chí Phèo mới có số phận bi thảm</x:v>
+      </x:c>
+      <x:c r="N6" s="27" t="str">
+        <x:v>Xã hội cũ đã đẩy nhiều người vào con đường xấu</x:v>
+      </x:c>
+      <x:c r="O6" s="27" t="str">
+        <x:v>Cả A và C</x:v>
+      </x:c>
+      <x:c r="P6" s="27" t="str"/>
+      <x:c r="Q6" s="27" t="str"/>
+      <x:c r="R6" s="27" t="str"/>
+    </x:row>
+    <x:row r="7" ht="54" customHeight="1">
       <x:c r="A7" s="27" t="str">
         <x:v>Demo/Cloze</x:v>
       </x:c>
       <x:c r="B7" s="27" t="str">
-        <x:v>CLZ_TABLE_001</x:v>
+        <x:v>CLZ_TABLE_002</x:v>
       </x:c>
       <x:c r="C7" s="27" t="str">
         <x:v>cloze</x:v>
       </x:c>
       <x:c r="D7" s="27" t="str">
-        <x:v>Một câu Cloze nhập từng dòng</x:v>
-      </x:c>
-      <x:c r="E7" s="27" t="str">
-        <x:v>Chọn đáp án hiển thị ngang.</x:v>
-      </x:c>
-      <x:c r="F7" s="27" t="str">
-        <x:v>mch</x:v>
-      </x:c>
+        <x:v>Một câu Cloze không có đoạn văn</x:v>
+      </x:c>
+      <x:c r="E7" s="27" t="str"/>
+      <x:c r="F7" s="27" t="str"/>
       <x:c r="G7" s="27" t="str">
-        <x:v>C</x:v>
+        <x:v>The capital of Vietnam is [[answer]].</x:v>
       </x:c>
       <x:c r="H7" s="27" t="str">
-        <x:v>a. Sai</x:v>
+        <x:v>shortanswer</x:v>
       </x:c>
       <x:c r="I7" s="27" t="str">
-        <x:v>b. Cũng sai</x:v>
+        <x:v>FALSE</x:v>
       </x:c>
       <x:c r="J7" s="27" t="str">
-        <x:v>c. Đúng</x:v>
+        <x:v>TRUE</x:v>
       </x:c>
       <x:c r="K7" s="27" t="str">
-        <x:v>d. Nửa đúng</x:v>
+        <x:v>Hanoi;Ha Noi</x:v>
       </x:c>
       <x:c r="L7" s="27" t="str"/>
-      <x:c r="M7" s="27" t="str">
-        <x:v>Sinh MCH, Moodle hiển thị lựa chọn dạng ngang.</x:v>
-      </x:c>
+      <x:c r="M7" s="27" t="str"/>
       <x:c r="N7" s="27" t="str"/>
-    </x:row>
-    <x:row r="8" ht="46" customHeight="1">
+      <x:c r="O7" s="27" t="str"/>
+      <x:c r="P7" s="27" t="str"/>
+      <x:c r="Q7" s="27" t="str">
+        <x:v>Có thể đặt [[answer]] để app chèn ô trả lời đúng vị trí.</x:v>
+      </x:c>
+      <x:c r="R7" s="27" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="54" customHeight="1">
       <x:c r="A8" s="27" t="str">
         <x:v>Demo/Cloze</x:v>
       </x:c>
       <x:c r="B8" s="27" t="str">
-        <x:v>CLZ_TABLE_001</x:v>
+        <x:v>CLZ_TABLE_002</x:v>
       </x:c>
       <x:c r="C8" s="27" t="str">
         <x:v>cloze</x:v>
       </x:c>
       <x:c r="D8" s="27" t="str">
-        <x:v>Một câu Cloze nhập từng dòng</x:v>
-      </x:c>
-      <x:c r="E8" s="27" t="str">
-        <x:v>Với công thức \(S=\pi r^2\), hằng số cần điền là gì?</x:v>
-      </x:c>
-      <x:c r="F8" s="27" t="str">
-        <x:v>shortanswer</x:v>
-      </x:c>
+        <x:v>Một câu Cloze không có đoạn văn</x:v>
+      </x:c>
+      <x:c r="E8" s="27" t="str"/>
+      <x:c r="F8" s="27" t="str"/>
       <x:c r="G8" s="27" t="str">
-        <x:v>pi</x:v>
-      </x:c>
-      <x:c r="H8" s="27" t="str"/>
-      <x:c r="I8" s="27" t="str"/>
-      <x:c r="J8" s="27" t="str"/>
-      <x:c r="K8" s="27" t="str"/>
+        <x:v>2 + 3 = [[answer]].</x:v>
+      </x:c>
+      <x:c r="H8" s="27" t="str">
+        <x:v>numerical</x:v>
+      </x:c>
+      <x:c r="I8" s="27" t="str">
+        <x:v>FALSE</x:v>
+      </x:c>
+      <x:c r="J8" s="27" t="str">
+        <x:v>TRUE</x:v>
+      </x:c>
+      <x:c r="K8" s="27" t="n">
+        <x:v>5</x:v>
+      </x:c>
       <x:c r="L8" s="27" t="str"/>
-      <x:c r="M8" s="27" t="str">
-        <x:v>Có thể viết LaTeX trong question_text.</x:v>
-      </x:c>
+      <x:c r="M8" s="27" t="str"/>
       <x:c r="N8" s="27" t="str"/>
-    </x:row>
-    <x:row r="9" ht="46" customHeight="1">
+      <x:c r="O8" s="27" t="str"/>
+      <x:c r="P8" s="27" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q8" s="27" t="str"/>
+      <x:c r="R8" s="27" t="str"/>
+    </x:row>
+    <x:row r="9" ht="54" customHeight="1">
       <x:c r="A9" s="27" t="str">
         <x:v>Demo/Cloze</x:v>
       </x:c>
@@ -2087,41 +2225,61 @@
         <x:v>cloze</x:v>
       </x:c>
       <x:c r="D9" s="27" t="str">
-        <x:v>Một câu Cloze khác</x:v>
-      </x:c>
-      <x:c r="E9" s="27" t="str">
-        <x:v>The capital of Vietnam is [[answer]].</x:v>
-      </x:c>
-      <x:c r="F9" s="27" t="str">
-        <x:v>shortanswer</x:v>
-      </x:c>
+        <x:v>Một câu Cloze không có đoạn văn</x:v>
+      </x:c>
+      <x:c r="E9" s="27" t="str"/>
+      <x:c r="F9" s="27" t="str"/>
       <x:c r="G9" s="27" t="str">
-        <x:v>Hanoi;Ha Noi</x:v>
-      </x:c>
-      <x:c r="H9" s="27" t="str"/>
-      <x:c r="I9" s="27" t="str"/>
-      <x:c r="J9" s="27" t="str"/>
-      <x:c r="K9" s="27" t="str"/>
-      <x:c r="L9" s="27" t="str"/>
+        <x:v>Số 7 thuộc loại nào?</x:v>
+      </x:c>
+      <x:c r="H9" s="27" t="str">
+        <x:v>mch</x:v>
+      </x:c>
+      <x:c r="I9" s="27" t="str">
+        <x:v>TRUE</x:v>
+      </x:c>
+      <x:c r="J9" s="27" t="str">
+        <x:v>TRUE</x:v>
+      </x:c>
+      <x:c r="K9" s="27" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="L9" s="27" t="str">
+        <x:v>Số nguyên tố</x:v>
+      </x:c>
       <x:c r="M9" s="27" t="str">
-        <x:v>Có thể đặt [[answer]] để app chèn ô trả lời đúng vị trí.</x:v>
-      </x:c>
-      <x:c r="N9" s="27" t="n">
-        <x:v>1</x:v>
-      </x:c>
+        <x:v>Số chẵn</x:v>
+      </x:c>
+      <x:c r="N9" s="27" t="str">
+        <x:v>Số âm</x:v>
+      </x:c>
+      <x:c r="O9" s="27" t="str">
+        <x:v>Hợp số</x:v>
+      </x:c>
+      <x:c r="P9" s="27" t="str"/>
+      <x:c r="Q9" s="27" t="str">
+        <x:v>Ví dụ MCH có đảo đáp án.</x:v>
+      </x:c>
+      <x:c r="R9" s="27" t="str"/>
     </x:row>
   </x:sheetData>
-  <x:dataValidations count="2">
+  <x:dataValidations count="4">
     <x:dataValidation type="list" sqref="C2:C200">
       <x:formula1>_Allowed_Values!$A$2:$A$12</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="F2:F200">
       <x:formula1>"shortanswer,shortanswer_c,numerical,multichoice,mcv,mch"</x:formula1>
     </x:dataValidation>
+    <x:dataValidation type="list" sqref="H2:H200">
+      <x:formula1>"shortanswer,shortanswer_c,numerical,multichoice,mcv,mch"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="I2:J200">
+      <x:formula1>"TRUE,FALSE"</x:formula1>
+    </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re2187623a8044b88"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc1cf092b98574c0b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2216,23 +2374,23 @@
         <x:v>cloze</x:v>
       </x:c>
       <x:c r="B12" s="12" t="str">
-        <x:v>Có thể nhập sẵn cú pháp Embedded answers trong question_text, hoặc nhập dạng bảng nhiều dòng cùng question_id. cloze_answer_type hỗ trợ: shortanswer, shortanswer_c, numerical, multichoice, mcv, mch. App sẽ tự sinh mã SHORTANSWER/SHORTANSWER_C/NUMERICAL/MULTICHOICE/MCV/MCH.</x:v>
+        <x:v>Có thể nhập sẵn cú pháp Embedded answers trong question_text, hoặc nhập dạng bảng nhiều dòng cùng question_id. Nếu có đoạn văn đọc hiểu, nhập passage_text ở dòng đầu của nhóm question_id; app sẽ đặt đoạn văn trước các câu hỏi nhỏ trong cùng câu Cloze. cloze_answer_type hỗ trợ: shortanswer, shortanswer_c, numerical, multichoice, mcv, mch.</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
-      <x:c r="A13" s="12" t="str">
-        <x:v>dragdrop_text</x:v>
-      </x:c>
-      <x:c r="B13" s="12" t="str">
-        <x:v>question_text phải chứa [[1]], [[2]], ...; mỗi dòng khai báo drag_no + drag_text. drag_no không có trong text sẽ là đáp án nhiễu.</x:v>
+      <x:c r="A13" s="57" t="str">
+        <x:v>shuffle_answers</x:v>
+      </x:c>
+      <x:c r="B13" s="27" t="str">
+        <x:v>TRUE de dao dap an; voi Cloze app se sinh MULTICHOICE_S/MCVS/MCHS.</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
-      <x:c r="A14" s="12" t="str">
-        <x:v>select_missing_words</x:v>
-      </x:c>
-      <x:c r="B14" s="12" t="str">
-        <x:v>Tương tự dragdrop_text nhưng Moodle hiển thị dạng hộp chọn thả xuống, xuất XML type gapselect.</x:v>
+      <x:c r="A14" s="57" t="str">
+        <x:v>show_correct_when_wrong</x:v>
+      </x:c>
+      <x:c r="B14" s="27" t="str">
+        <x:v>TRUE de chi hien 'Dap an dung' khi nguoi hoc chon sai tung o Cloze.</x:v>
       </x:c>
     </x:row>
     <x:row r="15">

</xml_diff>

<commit_message>
feat: add auto explanation support to cloze items and update related parsing logic
</commit_message>
<xml_diff>
--- a/public/templates/moodle_xml_sheet_templates.xlsx
+++ b/public/templates/moodle_xml_sheet_templates.xlsx
@@ -2,20 +2,20 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Allowed_Values" sheetId="1" r:id="Rcec0a542981e40d0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Huong_Dan" sheetId="2" r:id="R62aa9b46b6ae4da6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_Single_Choice" sheetId="3" r:id="R436118ae4f1f48fc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_Multiple_Choice" sheetId="4" r:id="Rd6742cd6601e47ac"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_TrueFalse" sheetId="5" r:id="R0d789be7aec04d22"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_ShortAnswer" sheetId="6" r:id="R3ab26ada3ee14149"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_Numerical" sheetId="7" r:id="Radf0e633a977447f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_Matching" sheetId="8" r:id="Rfbcc500d38a346c1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_DragDrop_Text" sheetId="9" r:id="Rae573c0837774eca"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_Essay_Desc_Cloze" sheetId="10" r:id="R3401de5ebee54700"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_Reading_Passage" sheetId="11" r:id="Rdda0ec4411314db2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_Full_Demo" sheetId="12" r:id="Rf27e5f82d7854367"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_Select_Missing_Words" sheetId="13" r:id="R2b1fb838d15b40b6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12_Cloze_Many_In_One" sheetId="14" r:id="R468f589aa0de43b8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Allowed_Values" sheetId="1" r:id="R4ba12024ac02434b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Huong_Dan" sheetId="2" r:id="R680ee7bb447a4dae"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_Single_Choice" sheetId="3" r:id="Ra12b275e09904c59"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_Multiple_Choice" sheetId="4" r:id="Rc14732a8b5fe4089"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_TrueFalse" sheetId="5" r:id="Ra29e743ee4cd4024"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_ShortAnswer" sheetId="6" r:id="Rae04d9f08f2145c1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_Numerical" sheetId="7" r:id="Rc4608a7c35754fbb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_Matching" sheetId="8" r:id="R05870fe521344812"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_DragDrop_Text" sheetId="9" r:id="R0f2b862126bf456a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_Essay_Desc_Cloze" sheetId="10" r:id="R4d246655a4d24ea3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_Reading_Passage" sheetId="11" r:id="R4f34b3506aa24dfb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_Full_Demo" sheetId="12" r:id="Rf785270231a44a5d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_Select_Missing_Words" sheetId="13" r:id="R27049b66d42242b4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12_Cloze_Many_In_One" sheetId="14" r:id="Re0a0fc258c594bfc"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -49,7 +49,7 @@
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="15">
+  <x:fills count="17">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -121,6 +121,16 @@
         <x:fgColor rgb="FFE2F0D9"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F4E78"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE2F0D9"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="3">
     <x:border/>
@@ -143,7 +153,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="58">
+  <x:cellXfs count="65">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -266,6 +276,23 @@
       <x:alignment wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="3" fillId="14" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="15" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="16" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -1802,7 +1829,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6d8d32c9c6434114"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf0a60648152c4aa3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1821,7 +1848,7 @@
     <x:col min="8" max="8" width="18" hidden="0" customWidth="1"/>
     <x:col min="9" max="9" width="18" hidden="0" customWidth="1"/>
     <x:col min="10" max="10" width="18" hidden="0" customWidth="1"/>
-    <x:col min="11" max="11" width="30" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="18" hidden="0" customWidth="1"/>
     <x:col min="12" max="12" width="30" hidden="0" customWidth="1"/>
     <x:col min="13" max="13" width="30" hidden="0" customWidth="1"/>
     <x:col min="14" max="14" width="30" hidden="0" customWidth="1"/>
@@ -1831,58 +1858,61 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1">
-      <x:c r="A1" s="51" t="str">
+      <x:c r="A1" s="58" t="str">
         <x:v>category</x:v>
       </x:c>
-      <x:c r="B1" s="51" t="str">
+      <x:c r="B1" s="58" t="str">
         <x:v>question_id</x:v>
       </x:c>
-      <x:c r="C1" s="51" t="str">
+      <x:c r="C1" s="58" t="str">
         <x:v>type</x:v>
       </x:c>
-      <x:c r="D1" s="51" t="str">
+      <x:c r="D1" s="58" t="str">
         <x:v>question_name</x:v>
       </x:c>
-      <x:c r="E1" s="51" t="str">
+      <x:c r="E1" s="58" t="str">
         <x:v>passage_id</x:v>
       </x:c>
-      <x:c r="F1" s="51" t="str">
+      <x:c r="F1" s="58" t="str">
         <x:v>passage_text</x:v>
       </x:c>
-      <x:c r="G1" s="51" t="str">
+      <x:c r="G1" s="58" t="str">
         <x:v>question_text</x:v>
       </x:c>
-      <x:c r="H1" s="51" t="str">
+      <x:c r="H1" s="58" t="str">
         <x:v>cloze_answer_type</x:v>
       </x:c>
-      <x:c r="I1" s="51" t="str">
+      <x:c r="I1" s="58" t="str">
         <x:v>shuffle_answers</x:v>
       </x:c>
-      <x:c r="J1" s="51" t="str">
+      <x:c r="J1" s="58" t="str">
         <x:v>show_correct_when_wrong</x:v>
       </x:c>
-      <x:c r="K1" s="51" t="str">
+      <x:c r="K1" s="58" t="str">
+        <x:v>auto_explanation</x:v>
+      </x:c>
+      <x:c r="L1" s="58" t="str">
         <x:v>correct_answer</x:v>
       </x:c>
-      <x:c r="L1" s="51" t="str">
+      <x:c r="M1" s="58" t="str">
         <x:v>option_a</x:v>
       </x:c>
-      <x:c r="M1" s="51" t="str">
+      <x:c r="N1" s="58" t="str">
         <x:v>option_b</x:v>
       </x:c>
-      <x:c r="N1" s="51" t="str">
+      <x:c r="O1" s="58" t="str">
         <x:v>option_c</x:v>
       </x:c>
-      <x:c r="O1" s="51" t="str">
+      <x:c r="P1" s="58" t="str">
         <x:v>option_d</x:v>
       </x:c>
-      <x:c r="P1" s="51" t="str">
+      <x:c r="Q1" s="58" t="str">
         <x:v>tolerance</x:v>
       </x:c>
-      <x:c r="Q1" s="51" t="str">
+      <x:c r="R1" s="58" t="str">
         <x:v>explanation</x:v>
       </x:c>
-      <x:c r="R1" s="51" t="str">
+      <x:c r="S1" s="58" t="str">
         <x:v>grade</x:v>
       </x:c>
     </x:row>
@@ -1918,25 +1948,28 @@
         <x:v>TRUE</x:v>
       </x:c>
       <x:c r="K2" s="27" t="str">
+        <x:v>FALSE</x:v>
+      </x:c>
+      <x:c r="L2" s="27" t="str">
         <x:v>B</x:v>
       </x:c>
-      <x:c r="L2" s="27" t="str">
+      <x:c r="M2" s="27" t="str">
         <x:v>1915</x:v>
       </x:c>
-      <x:c r="M2" s="27" t="str">
+      <x:c r="N2" s="27" t="str">
         <x:v>1917</x:v>
       </x:c>
-      <x:c r="N2" s="27" t="str">
+      <x:c r="O2" s="27" t="str">
         <x:v>1919</x:v>
       </x:c>
-      <x:c r="O2" s="27" t="str">
+      <x:c r="P2" s="27" t="str">
         <x:v>1921</x:v>
       </x:c>
-      <x:c r="P2" s="27" t="str"/>
-      <x:c r="Q2" s="27" t="str">
+      <x:c r="Q2" s="27"/>
+      <x:c r="R2" s="27" t="str">
         <x:v>Nếu chọn sai, Moodle sẽ hiện đáp án đúng cho riêng câu nhỏ này.</x:v>
       </x:c>
-      <x:c r="R2" s="27" t="n">
+      <x:c r="S2" s="27" t="n">
         <x:v>7</x:v>
       </x:c>
     </x:row>
@@ -1956,7 +1989,7 @@
       <x:c r="E3" s="27" t="str">
         <x:v>NC001</x:v>
       </x:c>
-      <x:c r="F3" s="27" t="str"/>
+      <x:c r="F3" s="27"/>
       <x:c r="G3" s="27" t="str">
         <x:v>Ý chính của đoạn văn là gì?</x:v>
       </x:c>
@@ -1970,23 +2003,26 @@
         <x:v>TRUE</x:v>
       </x:c>
       <x:c r="K3" s="27" t="str">
+        <x:v>FALSE</x:v>
+      </x:c>
+      <x:c r="L3" s="27" t="str">
         <x:v>A</x:v>
       </x:c>
-      <x:c r="L3" s="27" t="str">
+      <x:c r="M3" s="27" t="str">
         <x:v>Nam Cao là nhà văn hiện thực xuất sắc với những tác phẩm có giá trị</x:v>
       </x:c>
-      <x:c r="M3" s="27" t="str">
+      <x:c r="N3" s="27" t="str">
         <x:v>Chí Phèo là tác phẩm nổi tiếng nhất của Nam Cao</x:v>
       </x:c>
-      <x:c r="N3" s="27" t="str">
+      <x:c r="O3" s="27" t="str">
         <x:v>Nam Cao viết về người nông dân</x:v>
       </x:c>
-      <x:c r="O3" s="27" t="str">
+      <x:c r="P3" s="27" t="str">
         <x:v>Sự nghiệp sáng tác của Nam Cao không dài</x:v>
       </x:c>
-      <x:c r="P3" s="27" t="str"/>
-      <x:c r="Q3" s="27" t="str"/>
-      <x:c r="R3" s="27" t="str"/>
+      <x:c r="Q3" s="27"/>
+      <x:c r="R3" s="27"/>
+      <x:c r="S3" s="27"/>
     </x:row>
     <x:row r="4" ht="54" customHeight="1">
       <x:c r="A4" s="27" t="str">
@@ -2004,7 +2040,7 @@
       <x:c r="E4" s="27" t="str">
         <x:v>NC001</x:v>
       </x:c>
-      <x:c r="F4" s="27" t="str"/>
+      <x:c r="F4" s="27"/>
       <x:c r="G4" s="27" t="str">
         <x:v>Điều gì có thể suy ra từ đoạn văn?</x:v>
       </x:c>
@@ -2018,23 +2054,26 @@
         <x:v>TRUE</x:v>
       </x:c>
       <x:c r="K4" s="27" t="str">
+        <x:v>FALSE</x:v>
+      </x:c>
+      <x:c r="L4" s="27" t="str">
         <x:v>B</x:v>
       </x:c>
-      <x:c r="L4" s="27" t="str">
+      <x:c r="M4" s="27" t="str">
         <x:v>Nam Cao chỉ viết về người nông dân</x:v>
       </x:c>
-      <x:c r="M4" s="27" t="str">
+      <x:c r="N4" s="27" t="str">
         <x:v>Nam Cao quan tâm đến số phận người nông dân trong xã hội cũ</x:v>
       </x:c>
-      <x:c r="N4" s="27" t="str">
+      <x:c r="O4" s="27" t="str">
         <x:v>Nam Cao là nhà văn duy nhất viết về nông dân</x:v>
       </x:c>
-      <x:c r="O4" s="27" t="str">
+      <x:c r="P4" s="27" t="str">
         <x:v>Các tác phẩm của Nam Cao đã mất giá trị</x:v>
       </x:c>
-      <x:c r="P4" s="27" t="str"/>
-      <x:c r="Q4" s="27" t="str"/>
-      <x:c r="R4" s="27" t="str"/>
+      <x:c r="Q4" s="27"/>
+      <x:c r="R4" s="27"/>
+      <x:c r="S4" s="27"/>
     </x:row>
     <x:row r="5" ht="54" customHeight="1">
       <x:c r="A5" s="27" t="str">
@@ -2052,7 +2091,7 @@
       <x:c r="E5" s="27" t="str">
         <x:v>NC001</x:v>
       </x:c>
-      <x:c r="F5" s="27" t="str"/>
+      <x:c r="F5" s="27"/>
       <x:c r="G5" s="27" t="str">
         <x:v>Từ tha hóa trong đoạn văn có nghĩa gần nhất với từ nào?</x:v>
       </x:c>
@@ -2066,23 +2105,26 @@
         <x:v>TRUE</x:v>
       </x:c>
       <x:c r="K5" s="27" t="str">
+        <x:v>FALSE</x:v>
+      </x:c>
+      <x:c r="L5" s="27" t="str">
         <x:v>A</x:v>
       </x:c>
-      <x:c r="L5" s="27" t="str">
+      <x:c r="M5" s="27" t="str">
         <x:v>Suy thoái nhân phẩm</x:v>
       </x:c>
-      <x:c r="M5" s="27" t="str">
+      <x:c r="N5" s="27" t="str">
         <x:v>Trở nên giàu có</x:v>
       </x:c>
-      <x:c r="N5" s="27" t="str">
+      <x:c r="O5" s="27" t="str">
         <x:v>Bị bệnh tật</x:v>
       </x:c>
-      <x:c r="O5" s="27" t="str">
+      <x:c r="P5" s="27" t="str">
         <x:v>Mất nhà cửa</x:v>
       </x:c>
-      <x:c r="P5" s="27" t="str"/>
-      <x:c r="Q5" s="27" t="str"/>
-      <x:c r="R5" s="27" t="str"/>
+      <x:c r="Q5" s="27"/>
+      <x:c r="R5" s="27"/>
+      <x:c r="S5" s="27"/>
     </x:row>
     <x:row r="6" ht="54" customHeight="1">
       <x:c r="A6" s="27" t="str">
@@ -2100,7 +2142,7 @@
       <x:c r="E6" s="27" t="str">
         <x:v>NC001</x:v>
       </x:c>
-      <x:c r="F6" s="27" t="str"/>
+      <x:c r="F6" s="27"/>
       <x:c r="G6" s="27" t="str">
         <x:v>Câu Đó không chỉ là số phận của một người mà là số phận của cả một tầng lớp trong xã hội cũ có ý nghĩa gì?</x:v>
       </x:c>
@@ -2114,23 +2156,26 @@
         <x:v>TRUE</x:v>
       </x:c>
       <x:c r="K6" s="27" t="str">
+        <x:v>FALSE</x:v>
+      </x:c>
+      <x:c r="L6" s="27" t="str">
         <x:v>D</x:v>
       </x:c>
-      <x:c r="L6" s="27" t="str">
+      <x:c r="M6" s="27" t="str">
         <x:v>Chí Phèo đại diện cho số phận của nhiều người trong xã hội cũ</x:v>
       </x:c>
-      <x:c r="M6" s="27" t="str">
+      <x:c r="N6" s="27" t="str">
         <x:v>Chỉ có Chí Phèo mới có số phận bi thảm</x:v>
       </x:c>
-      <x:c r="N6" s="27" t="str">
+      <x:c r="O6" s="27" t="str">
         <x:v>Xã hội cũ đã đẩy nhiều người vào con đường xấu</x:v>
       </x:c>
-      <x:c r="O6" s="27" t="str">
+      <x:c r="P6" s="27" t="str">
         <x:v>Cả A và C</x:v>
       </x:c>
-      <x:c r="P6" s="27" t="str"/>
-      <x:c r="Q6" s="27" t="str"/>
-      <x:c r="R6" s="27" t="str"/>
+      <x:c r="Q6" s="27"/>
+      <x:c r="R6" s="27"/>
+      <x:c r="S6" s="27"/>
     </x:row>
     <x:row r="7" ht="54" customHeight="1">
       <x:c r="A7" s="27" t="str">
@@ -2145,8 +2190,8 @@
       <x:c r="D7" s="27" t="str">
         <x:v>Một câu Cloze không có đoạn văn</x:v>
       </x:c>
-      <x:c r="E7" s="27" t="str"/>
-      <x:c r="F7" s="27" t="str"/>
+      <x:c r="E7" s="27"/>
+      <x:c r="F7" s="27"/>
       <x:c r="G7" s="27" t="str">
         <x:v>The capital of Vietnam is [[answer]].</x:v>
       </x:c>
@@ -2154,23 +2199,26 @@
         <x:v>shortanswer</x:v>
       </x:c>
       <x:c r="I7" s="27" t="str">
-        <x:v>FALSE</x:v>
+        <x:v>TRUE</x:v>
       </x:c>
       <x:c r="J7" s="27" t="str">
         <x:v>TRUE</x:v>
       </x:c>
       <x:c r="K7" s="27" t="str">
+        <x:v>FALSE</x:v>
+      </x:c>
+      <x:c r="L7" s="27" t="str">
         <x:v>Hanoi;Ha Noi</x:v>
       </x:c>
-      <x:c r="L7" s="27" t="str"/>
-      <x:c r="M7" s="27" t="str"/>
-      <x:c r="N7" s="27" t="str"/>
-      <x:c r="O7" s="27" t="str"/>
-      <x:c r="P7" s="27" t="str"/>
-      <x:c r="Q7" s="27" t="str">
+      <x:c r="M7" s="27"/>
+      <x:c r="N7" s="27"/>
+      <x:c r="O7" s="27"/>
+      <x:c r="P7" s="27"/>
+      <x:c r="Q7" s="27"/>
+      <x:c r="R7" s="27" t="str">
         <x:v>Có thể đặt [[answer]] để app chèn ô trả lời đúng vị trí.</x:v>
       </x:c>
-      <x:c r="R7" s="27" t="n">
+      <x:c r="S7" s="27" t="n">
         <x:v>1</x:v>
       </x:c>
     </x:row>
@@ -2187,8 +2235,8 @@
       <x:c r="D8" s="27" t="str">
         <x:v>Một câu Cloze không có đoạn văn</x:v>
       </x:c>
-      <x:c r="E8" s="27" t="str"/>
-      <x:c r="F8" s="27" t="str"/>
+      <x:c r="E8" s="27"/>
+      <x:c r="F8" s="27"/>
       <x:c r="G8" s="27" t="str">
         <x:v>2 + 3 = [[answer]].</x:v>
       </x:c>
@@ -2196,23 +2244,26 @@
         <x:v>numerical</x:v>
       </x:c>
       <x:c r="I8" s="27" t="str">
-        <x:v>FALSE</x:v>
+        <x:v>TRUE</x:v>
       </x:c>
       <x:c r="J8" s="27" t="str">
         <x:v>TRUE</x:v>
       </x:c>
-      <x:c r="K8" s="27" t="n">
+      <x:c r="K8" s="27" t="str">
+        <x:v>FALSE</x:v>
+      </x:c>
+      <x:c r="L8" s="27" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="L8" s="27" t="str"/>
-      <x:c r="M8" s="27" t="str"/>
-      <x:c r="N8" s="27" t="str"/>
-      <x:c r="O8" s="27" t="str"/>
-      <x:c r="P8" s="27" t="n">
+      <x:c r="M8" s="27"/>
+      <x:c r="N8" s="27"/>
+      <x:c r="O8" s="27"/>
+      <x:c r="P8" s="27"/>
+      <x:c r="Q8" s="27" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="Q8" s="27" t="str"/>
-      <x:c r="R8" s="27" t="str"/>
+      <x:c r="R8" s="27"/>
+      <x:c r="S8" s="27"/>
     </x:row>
     <x:row r="9" ht="54" customHeight="1">
       <x:c r="A9" s="27" t="str">
@@ -2227,8 +2278,8 @@
       <x:c r="D9" s="27" t="str">
         <x:v>Một câu Cloze không có đoạn văn</x:v>
       </x:c>
-      <x:c r="E9" s="27" t="str"/>
-      <x:c r="F9" s="27" t="str"/>
+      <x:c r="E9" s="27"/>
+      <x:c r="F9" s="27"/>
       <x:c r="G9" s="27" t="str">
         <x:v>Số 7 thuộc loại nào?</x:v>
       </x:c>
@@ -2242,28 +2293,31 @@
         <x:v>TRUE</x:v>
       </x:c>
       <x:c r="K9" s="27" t="str">
+        <x:v>FALSE</x:v>
+      </x:c>
+      <x:c r="L9" s="27" t="str">
         <x:v>A</x:v>
       </x:c>
-      <x:c r="L9" s="27" t="str">
+      <x:c r="M9" s="27" t="str">
         <x:v>Số nguyên tố</x:v>
       </x:c>
-      <x:c r="M9" s="27" t="str">
+      <x:c r="N9" s="27" t="str">
         <x:v>Số chẵn</x:v>
       </x:c>
-      <x:c r="N9" s="27" t="str">
+      <x:c r="O9" s="27" t="str">
         <x:v>Số âm</x:v>
       </x:c>
-      <x:c r="O9" s="27" t="str">
+      <x:c r="P9" s="27" t="str">
         <x:v>Hợp số</x:v>
       </x:c>
-      <x:c r="P9" s="27" t="str"/>
-      <x:c r="Q9" s="27" t="str">
+      <x:c r="Q9" s="27"/>
+      <x:c r="R9" s="27" t="str">
         <x:v>Ví dụ MCH có đảo đáp án.</x:v>
       </x:c>
-      <x:c r="R9" s="27" t="str"/>
+      <x:c r="S9" s="27"/>
     </x:row>
   </x:sheetData>
-  <x:dataValidations count="4">
+  <x:dataValidations count="7">
     <x:dataValidation type="list" sqref="C2:C200">
       <x:formula1>_Allowed_Values!$A$2:$A$12</x:formula1>
     </x:dataValidation>
@@ -2276,10 +2330,19 @@
     <x:dataValidation type="list" sqref="I2:J200">
       <x:formula1>"TRUE,FALSE"</x:formula1>
     </x:dataValidation>
+    <x:dataValidation type="list" sqref="I2:J9">
+      <x:formula1>"TRUE,FALSE"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="K2:K200">
+      <x:formula1>"TRUE,FALSE"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="I2:K200">
+      <x:formula1>"TRUE,FALSE"</x:formula1>
+    </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc1cf092b98574c0b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raeec7536486446fc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2394,11 +2457,11 @@
       </x:c>
     </x:row>
     <x:row r="15">
-      <x:c r="A15" s="12" t="str">
-        <x:v>unlimited</x:v>
-      </x:c>
-      <x:c r="B15" s="12" t="str">
-        <x:v>TRUE nếu lựa chọn kéo-thả được dùng lại nhiều lần; FALSE hoặc bỏ trống nếu không.</x:v>
+      <x:c r="A15" s="64" t="str">
+        <x:v>auto_explanation</x:v>
+      </x:c>
+      <x:c r="B15" s="27" t="str">
+        <x:v>TRUE de app tu sinh feedback ngan cho tung cau Cloze khi explanation trong sheet dang trong.</x:v>
       </x:c>
     </x:row>
     <x:row r="16">

</xml_diff>